<commit_message>
Add split-detection safeguards (S-001) + fix sub-floor WACCs for ABBV/PEP/KO/V
Engine:
- fmp_3statementv6.py: S-001 YoY share-count check in build_dcf() prints
  [S-001 WARNING] when shares move >25% YoY, flagging likely stock splits before
  they corrupt per-share multiples (zero extra FMP calls)

Rules:
- CLAUDE.md Rule 22: No Speculative Valuation Claims -- must fetch live FMP
  before stating any current price, mktcap, P/E, share count, or multiple in chat

Re-runs (WACC floor 8.5% now applied):
- ABBV 6.0->6.5 (raw WACC 6.82%), PEP 8.0->8.1 (6.91%), KO 6.0->6.1 (7.15%)
- V 7.4->6.2: WACC floored (raw 7.67%); Rule 15 fires (no P/E data) -- honest
- WMT: skipped (HTTP 429); re-run pending quota reset

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/excel/ABBV_model.xlsx
+++ b/static/excel/ABBV_model.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="P&amp;L" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Balance Sheet" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flow" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Ratios &amp; FCF" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Segments" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="WACC" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="DCF" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Scorecard" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;L" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ratios &amp; FCF" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WACC" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorecard" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7358,11 +7358,11 @@
         </is>
       </c>
       <c r="B5" s="43" t="n">
-        <v>372484.096487</v>
+        <v>381097.21149</v>
       </c>
       <c r="C5" s="44" t="inlineStr">
         <is>
-          <t>FMP marketCap  |  price $210.825</t>
+          <t>FMP marketCap  |  price $215.7</t>
         </is>
       </c>
     </row>
@@ -7444,11 +7444,11 @@
         </is>
       </c>
       <c r="B12" s="46" t="n">
-        <v>0.0446</v>
+        <v>0.0457</v>
       </c>
       <c r="C12" s="44" t="inlineStr">
         <is>
-          <t>FRED series DGS10  |  latest: 2026-05-13</t>
+          <t>FRED series DGS10  |  latest: 2026-05-21</t>
         </is>
       </c>
     </row>
@@ -7459,7 +7459,7 @@
         </is>
       </c>
       <c r="B13" s="48" t="n">
-        <v>0.0446</v>
+        <v>0.0457</v>
       </c>
       <c r="C13" s="49" t="inlineStr">
         <is>
@@ -7531,7 +7531,7 @@
         </is>
       </c>
       <c r="B19" s="50" t="n">
-        <v>1.118</v>
+        <v>1.115</v>
       </c>
       <c r="C19" s="44">
         <f> unlevered × (1 + (1 − t) × D/E)</f>
@@ -7545,7 +7545,7 @@
         </is>
       </c>
       <c r="B20" s="51" t="n">
-        <v>0.652</v>
+        <v>0.651</v>
       </c>
       <c r="C20" s="49" t="inlineStr">
         <is>
@@ -7719,11 +7719,11 @@
         </is>
       </c>
       <c r="B35" s="46" t="n">
-        <v>0.0554</v>
+        <v>0.05650000000000001</v>
       </c>
       <c r="C35" s="44" t="inlineStr">
         <is>
-          <t>Rf 4.46% + spread 1.08%</t>
+          <t>Rf 4.57% + spread 1.08%</t>
         </is>
       </c>
     </row>
@@ -7749,7 +7749,7 @@
         </is>
       </c>
       <c r="B37" s="48" t="n">
-        <v>0.0491</v>
+        <v>0.0496</v>
       </c>
       <c r="C37" s="49" t="inlineStr">
         <is>
@@ -7814,16 +7814,16 @@
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="54" t="inlineStr">
         <is>
-          <t>WACC  =  (E/V × Re)  +  (D/V × Rd × (1 − t))</t>
+          <t>WACC  =  MAX(8.5%, (E/V × Re) + (D/V × Rd × (1 − t)))</t>
         </is>
       </c>
       <c r="B44" s="55">
-        <f>B8*B28+B9*B37*(1-B41)</f>
+        <f>MAX(0.085, B8*B28+B9*B37*(1-B41))</f>
         <v/>
       </c>
       <c r="C44" s="56" t="inlineStr">
         <is>
-          <t>Used as discount rate in DCF tab</t>
+          <t>Floored 8.5% (D-001); raw formula below</t>
         </is>
       </c>
     </row>
@@ -8539,7 +8539,7 @@
         <v>67283.8</v>
       </c>
       <c r="H15" s="77" t="n">
-        <v>72633.7</v>
+        <v>72633.60000000001</v>
       </c>
       <c r="I15" s="77" t="n">
         <v>77836</v>
@@ -8570,27 +8570,27 @@
       </c>
       <c r="G16" s="82" t="inlineStr">
         <is>
-          <t>66,573 — 67,744</t>
+          <t>67,034 — 67,654</t>
         </is>
       </c>
       <c r="H16" s="82" t="inlineStr">
         <is>
-          <t>70,385 — 73,957</t>
+          <t>71,102 — 73,927</t>
         </is>
       </c>
       <c r="I16" s="82" t="inlineStr">
         <is>
-          <t>77,748 — 77,924</t>
+          <t>77,797 — 77,875</t>
         </is>
       </c>
       <c r="J16" s="82" t="inlineStr">
         <is>
-          <t>80,195 — 83,360</t>
+          <t>80,314 — 83,089</t>
         </is>
       </c>
       <c r="K16" s="82" t="inlineStr">
         <is>
-          <t>81,939 — 85,174</t>
+          <t>82,035 — 84,869</t>
         </is>
       </c>
       <c r="L16" s="83" t="inlineStr">
@@ -8614,16 +8614,16 @@
         <v>22</v>
       </c>
       <c r="H17" s="84" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I17" s="84" t="n">
+        <v>24</v>
+      </c>
+      <c r="J17" s="84" t="n">
         <v>23</v>
       </c>
-      <c r="J17" s="84" t="n">
-        <v>11</v>
-      </c>
       <c r="K17" s="84" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="L17" s="83" t="inlineStr">
         <is>
@@ -8734,7 +8734,7 @@
         <v/>
       </c>
       <c r="G20" s="77" t="n">
-        <v>23029</v>
+        <v>23029.1</v>
       </c>
       <c r="H20" s="77" t="n">
         <v>24860.1</v>
@@ -8768,27 +8768,27 @@
       </c>
       <c r="G21" s="82" t="inlineStr">
         <is>
-          <t>22,786 — 23,187</t>
+          <t>22,944 — 23,156</t>
         </is>
       </c>
       <c r="H21" s="82" t="inlineStr">
         <is>
-          <t>24,090 — 25,313</t>
+          <t>24,336 — 25,303</t>
         </is>
       </c>
       <c r="I21" s="82" t="inlineStr">
         <is>
-          <t>26,610 — 26,671</t>
+          <t>26,627 — 26,654</t>
         </is>
       </c>
       <c r="J21" s="82" t="inlineStr">
         <is>
-          <t>27,448 — 28,531</t>
+          <t>27,489 — 28,439</t>
         </is>
       </c>
       <c r="K21" s="82" t="inlineStr">
         <is>
-          <t>28,045 — 29,152</t>
+          <t>28,078 — 29,048</t>
         </is>
       </c>
       <c r="L21" s="83" t="inlineStr">
@@ -9452,7 +9452,7 @@
         </is>
       </c>
       <c r="B38" s="100" t="n">
-        <v>10</v>
+        <v>15.6</v>
       </c>
       <c r="C38" s="98" t="n"/>
       <c r="D38" s="98" t="n"/>
@@ -9466,7 +9466,7 @@
       <c r="L38" s="98" t="n"/>
       <c r="M38" s="74" t="inlineStr">
         <is>
-          <t>Growth tier: LOW (1.9% 3yr avg rev growth).  Bear 8x / Base 10x / Bull 12x.  Override manually if needed.</t>
+          <t>Growth tier: LOW (1.9% 3yr avg rev growth).  Bear 12x / Base 16x / Bull 19x.  Override manually if needed.</t>
         </is>
       </c>
     </row>
@@ -9968,7 +9968,7 @@
         </is>
       </c>
       <c r="B61" s="111" t="n">
-        <v>210.82</v>
+        <v>215.7</v>
       </c>
       <c r="C61" s="103" t="n"/>
       <c r="D61" s="103" t="n"/>
@@ -10068,7 +10068,7 @@
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="113" t="inlineStr">
         <is>
-          <t>JS SCORECARD — ABBV  |  Master Prompt v2  |  15 May 2026  |  Sector bucket: Stable Compounder</t>
+          <t>JS SCORECARD — ABBV  |  Master Prompt v2  |  25 May 2026  |  Sector bucket: Stable Compounder</t>
         </is>
       </c>
     </row>
@@ -10201,7 +10201,7 @@
       </c>
       <c r="D9" s="129" t="inlineStr">
         <is>
-          <t>GM 70.2% ✓ (&gt;40%)  |  GM trend +0.2% ✗ (&gt;+1pp)  |  ROIC-WACC +18.8% ✓ (&gt;+5pp)  |  Rev consistency σ=5.4% ✓ (&lt;8%)  [3/4 indicators positive — proxy score]</t>
+          <t>GM 70.2% ✓ (&gt;40%)  |  GM trend +0.2% ✗ (&gt;+1pp)  |  ROIC-WACC +16.3% ✓ (&gt;+5pp)  |  Rev consistency σ=5.4% ✓ (&lt;8%)  [3/4 indicators positive — proxy score]</t>
         </is>
       </c>
       <c r="E9" s="130" t="inlineStr">
@@ -10218,7 +10218,7 @@
       </c>
       <c r="H9" s="133" t="inlineStr">
         <is>
-          <t>GM 70.2% ✓ (&gt;40%)  |  GM trend +0.2% ✗ (&gt;+1pp)  |  ROIC-WACC +18.8% ✓ (&gt;+5pp)  |  Rev consistency σ=5.4% ✓ (&lt;8%)  [3/4 indicators positive — proxy score]</t>
+          <t>GM 70.2% ✓ (&gt;40%)  |  GM trend +0.2% ✗ (&gt;+1pp)  |  ROIC-WACC +16.3% ✓ (&gt;+5pp)  |  Rev consistency σ=5.4% ✓ (&lt;8%)  [3/4 indicators positive — proxy score]</t>
         </is>
       </c>
     </row>
@@ -10268,7 +10268,7 @@
       </c>
       <c r="D11" s="129" t="inlineStr">
         <is>
-          <t>ROIC trend -0.7% ✓ (≥-2pp)  |  GM maintained +0.2% ✓  |  Op margin +1.6% ✓ (≥-2pp)  |  Capital returns HIGH ✓  |  Share count +0.1%/yr ✓ (≤+2%/yr)  [5/5 indicators positive — proxy score]</t>
+          <t>ROIC trend -0.7% ✓ (&gt;=-2pp)  |  GM maintained +0.2% ✓  |  Op margin +1.6% ✓ (≥-2pp)  |  Capital returns HIGH ✓  |  Share count +0.1%/yr ✓ (≤+2%/yr)  [5/5 indicators positive — proxy score]</t>
         </is>
       </c>
       <c r="E11" s="134" t="inlineStr">
@@ -10285,7 +10285,7 @@
       </c>
       <c r="H11" s="133" t="inlineStr">
         <is>
-          <t>ROIC trend -0.7% ✓ (≥-2pp)  |  GM maintained +0.2% ✓  |  Op margin +1.6% ✓ (≥-2pp)  |  Capital returns HIGH ✓  |  Share count +0.1%/yr ✓ (≤+2%/yr)  [5/5 indicators positive — proxy score]</t>
+          <t>ROIC trend -0.7% ✓ (&gt;=-2pp)  |  GM maintained +0.2% ✓  |  Op margin +1.6% ✓ (≥-2pp)  |  Capital returns HIGH ✓  |  Share count +0.1%/yr ✓ (≤+2%/yr)  [5/5 indicators positive — proxy score]</t>
         </is>
       </c>
     </row>
@@ -10358,7 +10358,7 @@
         </is>
       </c>
       <c r="F14" s="131" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G14" s="132">
         <f>IF(F14="",0,C14*F14*10)</f>
@@ -10432,7 +10432,7 @@
         </is>
       </c>
       <c r="F16" s="131" t="n">
-        <v>10.33</v>
+        <v>10</v>
       </c>
       <c r="G16" s="132">
         <f>IF(F16="",0,C16*F16*10)</f>
@@ -10541,7 +10541,7 @@
       </c>
       <c r="D20" s="129" t="inlineStr">
         <is>
-          <t>Rev growth σ=5.4%  |  Op margin σ=6.4%  [proxy — lower σ = lower risk = higher score]</t>
+          <t>Rev growth σ=5.4%  |  OM trend +1.0%, σ=6.4%  [quality = direction + stability]</t>
         </is>
       </c>
       <c r="E20" s="136" t="inlineStr">
@@ -10550,7 +10550,7 @@
         </is>
       </c>
       <c r="F20" s="131" t="n">
-        <v>5</v>
+        <v>3.33</v>
       </c>
       <c r="G20" s="132">
         <f>IF(F20="",0,C20*F20*10)</f>
@@ -10558,7 +10558,7 @@
       </c>
       <c r="H20" s="133" t="inlineStr">
         <is>
-          <t>Rev growth σ=5.4%  |  Op margin σ=6.4%  [proxy — lower σ = lower risk = higher score]</t>
+          <t>Rev growth σ=5.4%  |  OM trend +1.0%, σ=6.4%  [quality = direction + stability]</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10585,7 @@
       </c>
       <c r="D22" s="129" t="inlineStr">
         <is>
-          <t>Current 96.3x  |  5yr avg 54.2x  |  DCF-implied 100.4x  [+78% vs benchmark]</t>
+          <t>Current 96.3x  |  5yr avg 54.2x  |  DCF-implied 66.9x [ref only — not used as benchmark]  [+78% vs benchmark]  [trail=0.00 | fwd_pe=15.1x→10.00 | abs=0.0 → blended 40/40/20=4.00]  PEG=3.02 (fwd_pe=15.1x / eps_growth=500%)  [revision:Strong upgrade cycle→+0.50]</t>
         </is>
       </c>
       <c r="E22" s="135" t="inlineStr">
@@ -10594,7 +10594,7 @@
         </is>
       </c>
       <c r="F22" s="131" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="G22" s="132">
         <f>IF(F22="",0,C22*F22*10)</f>
@@ -10602,7 +10602,7 @@
       </c>
       <c r="H22" s="133" t="inlineStr">
         <is>
-          <t>Current 96.3x  |  5yr avg 54.2x  |  DCF-implied 100.4x  [+78% vs benchmark]</t>
+          <t>Current 96.3x  |  5yr avg 54.2x  |  DCF-implied 66.9x [ref only — not used as benchmark]  [+78% vs benchmark]  [trail=0.00 | fwd_pe=15.1x→10.00 | abs=0.0 → blended 40/40/20=4.00]  PEG=3.02 (fwd_pe=15.1x / eps_growth=500%)  [revision:Strong upgrade cycle→+0.50]</t>
         </is>
       </c>
     </row>
@@ -10622,7 +10622,7 @@
       </c>
       <c r="D23" s="129" t="inlineStr">
         <is>
-          <t>Current 22.8x  |  5yr avg 15.1x  |  DCF-implied 23.8x  [+51% vs benchmark]</t>
+          <t>Current 22.8x  |  5yr avg 15.1x  |  DCF-implied 15.9x [ref only — not used as benchmark]  [+51% vs benchmark]  [trail=0.00 | fwd_pfcf=19.6x→2.42 | abs=7.5 → blended 40/40/20=2.47]  [fcf_yield=4.4% vs rf=4.6%  spread=-0.2%→modifier=-0.25]</t>
         </is>
       </c>
       <c r="E23" s="135" t="inlineStr">
@@ -10631,7 +10631,7 @@
         </is>
       </c>
       <c r="F23" s="131" t="n">
-        <v>0</v>
+        <v>2.22</v>
       </c>
       <c r="G23" s="132">
         <f>IF(F23="",0,C23*F23*10)</f>
@@ -10639,7 +10639,7 @@
       </c>
       <c r="H23" s="133" t="inlineStr">
         <is>
-          <t>Current 22.8x  |  5yr avg 15.1x  |  DCF-implied 23.8x  [+51% vs benchmark]</t>
+          <t>Current 22.8x  |  5yr avg 15.1x  |  DCF-implied 15.9x [ref only — not used as benchmark]  [+51% vs benchmark]  [trail=0.00 | fwd_pfcf=19.6x→2.42 | abs=7.5 → blended 40/40/20=2.47]  [fcf_yield=4.4% vs rf=4.6%  spread=-0.2%→modifier=-0.25]</t>
         </is>
       </c>
     </row>

</xml_diff>